<commit_message>
feat(gui): 支持 set/modify/remove 按引用单号区间生成 Excel
</commit_message>
<xml_diff>
--- a/data/set.xlsx
+++ b/data/set.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J108"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -435,7 +435,7 @@
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="17" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>S001</t>
+          <t>SG0001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>运行一个云单(Mode=1)</t>
+          <t>set 引用当日第 1 号</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -549,7 +549,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>S002</t>
+          <t>SG0002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>运行多个云单(Mode=1)</t>
+          <t>set 引用当日第 2 号</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -581,34 +581,32 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>__REF1__,__REF2__</t>
+          <t>__REF2__</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>两个真实引用</t>
+          <t>主用例：模板行，字段值勿改</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>S003</t>
+          <t>S005</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>probe</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>停止一个云单(Mode=0)</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
+          <t>正确账号 不带 Model</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>7</v>
       </c>
@@ -621,7 +619,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -630,24 +628,24 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>期望 Err&gt;=0, Mode=0</t>
+          <t>省略 Model，看是否必填</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>S004</t>
+          <t>S006</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>probe</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>停止多个云单(Mode=0)</t>
+          <t>正确账号 AccAtt=0(股票渠道)</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -657,7 +655,7 @@
         <v>7</v>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -665,36 +663,38 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>__REF1__,__REF2__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>两个真实引用</t>
+          <t>渠道变体</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S005</t>
+          <t>S101</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>probe</t>
+          <t>error</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>正确账号 不带 Model</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>Refs 为空</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
       <c r="E6" t="n">
         <v>7</v>
       </c>
@@ -709,31 +709,27 @@
       <c r="H6" t="n">
         <v>1</v>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>__REF1__</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>省略 Model，看是否必填</t>
+          <t>期望被拒绝/Err&lt;0</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>S006</t>
+          <t>S102</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>probe</t>
+          <t>error</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>正确账号 AccAtt=0(股票渠道)</t>
+          <t>Mode 非法值99</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -743,7 +739,7 @@
         <v>7</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -751,7 +747,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -760,14 +756,14 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>渠道变体</t>
+          <t>期望被拒绝/Err&lt;0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>S101</t>
+          <t>S103</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -777,7 +773,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Refs 为空</t>
+          <t>Refs 不存在</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -797,17 +793,21 @@
       <c r="H8" t="n">
         <v>1</v>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>20991231000000</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>期望被拒绝/Err&lt;0</t>
+          <t>云单不存在，期望 Err&lt;0</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>S102</t>
+          <t>S104</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Mode 非法值99</t>
+          <t>FAccount 为空</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -829,13 +829,9 @@
       <c r="F9" t="n">
         <v>6</v>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>010100011300</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -851,7 +847,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S103</t>
+          <t>S105</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -861,7 +857,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Refs 不存在</t>
+          <t>Mode 为空</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -878,24 +874,22 @@
           <t>010100011300</t>
         </is>
       </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>20991231000000</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>云单不存在，期望 Err&lt;0</t>
+          <t>Mode 缺失，期望被拒绝</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S104</t>
+          <t>S106</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -905,19 +899,23 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FAccount 为空</t>
+          <t>AccountType 非法值99</t>
         </is>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>99</v>
       </c>
       <c r="F11" t="n">
         <v>6</v>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>010100011300</t>
+        </is>
+      </c>
       <c r="H11" t="n">
         <v>1</v>
       </c>
@@ -935,17 +933,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S105</t>
+          <t>S201</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>destroy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Mode 为空</t>
+          <t>Refs 超长1000字符</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -962,39 +960,41 @@
           <t>010100011300</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__LONG__</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Mode 缺失，期望被拒绝</t>
+          <t>超长引用</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>S106</t>
+          <t>S202</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>destroy</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AccountType 非法值99</t>
+          <t>Refs 含控制字符</t>
         </is>
       </c>
       <c r="D13" t="n">
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>99</v>
+        <v>7</v>
       </c>
       <c r="F13" t="n">
         <v>6</v>
@@ -1009,19 +1009,19 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__CTRL__</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>期望被拒绝/Err&lt;0</t>
+          <t>控制字符</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>S201</t>
+          <t>S203</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Refs 超长1000字符</t>
+          <t>Mode 极大值</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1048,34 +1048,36 @@
           <t>010100011300</t>
         </is>
       </c>
-      <c r="H14" t="n">
-        <v>1</v>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>__MAXINT__</t>
+        </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>__LONG__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>超长引用</t>
+          <t>极大值</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>S202</t>
+          <t>E700</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>destroy</t>
+          <t>error</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Refs 含控制字符</t>
+          <t>Mode=99</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1093,33 +1095,33 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>__CTRL__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>控制字符</t>
+          <t>主用例：模板行，字段值勿改</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>S203</t>
+          <t>E701</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>destroy</t>
+          <t>error</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mode 极大值</t>
+          <t>Mode=-1</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1136,10 +1138,8 @@
           <t>010100011300</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>__MAXINT__</t>
-        </is>
+      <c r="H16" t="n">
+        <v>-1</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1148,14 +1148,14 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>极大值</t>
+          <t>主用例：模板行，字段值勿改</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>E700</t>
+          <t>E702</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Mode=99</t>
+          <t>Mode=0</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1199,7 +1199,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>E701</t>
+          <t>E703</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mode=-1</t>
+          <t>Mode='abc'</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1226,8 +1226,10 @@
           <t>010100011300</t>
         </is>
       </c>
-      <c r="H18" t="n">
-        <v>-1</v>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1243,7 +1245,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>E702</t>
+          <t>E704</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1253,7 +1255,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mode=0</t>
+          <t>Mode='__MAXINT__'</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1270,8 +1272,10 @@
           <t>010100011300</t>
         </is>
       </c>
-      <c r="H19" t="n">
-        <v>0</v>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>__MAXINT__</t>
+        </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1287,7 +1291,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>E703</t>
+          <t>E705</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1297,7 +1301,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mode='abc'</t>
+          <t>Mode='__HUGE__'</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1316,7 +1320,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>abc</t>
+          <t>__HUGE__</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1333,7 +1337,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>E704</t>
+          <t>E706</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1343,7 +1347,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Mode='__MAXINT__'</t>
+          <t>Mode='__HEX__'</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1362,7 +1366,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>__MAXINT__</t>
+          <t>__HEX__</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1379,7 +1383,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>E705</t>
+          <t>E707</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1389,7 +1393,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mode='__HUGE__'</t>
+          <t>Mode='__BOOL_WEIRD__'</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1408,7 +1412,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>__HUGE__</t>
+          <t>__BOOL_WEIRD__</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1425,7 +1429,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>E706</t>
+          <t>E708</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1435,7 +1439,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mode='__HEX__'</t>
+          <t>Refs=''</t>
         </is>
       </c>
       <c r="D23" t="n">
@@ -1452,16 +1456,10 @@
           <t>010100011300</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>__HEX__</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>__REF1__</t>
-        </is>
-      </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>主用例：模板行，字段值勿改</t>
@@ -1471,7 +1469,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>E707</t>
+          <t>E709</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1481,7 +1479,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mode='__BOOL_WEIRD__'</t>
+          <t>Refs='__SQL__'</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1498,14 +1496,12 @@
           <t>010100011300</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>__BOOL_WEIRD__</t>
-        </is>
+      <c r="H24" t="n">
+        <v>1</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__SQL__</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1517,7 +1513,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>E708</t>
+          <t>E710</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1527,7 +1523,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Refs=''</t>
+          <t>Refs='20991231000000'</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1547,7 +1543,11 @@
       <c r="H25" t="n">
         <v>1</v>
       </c>
-      <c r="I25" t="inlineStr"/>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>20991231000000</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
           <t>主用例：模板行，字段值勿改</t>
@@ -1557,7 +1557,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>E709</t>
+          <t>E711</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Refs='__SQL__'</t>
+          <t>Refs='__CTRL__'</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>__SQL__</t>
+          <t>__CTRL__</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1601,7 +1601,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>E710</t>
+          <t>E712</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Refs='20991231000000'</t>
+          <t>Refs='__EMOJI__'</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>20991231000000</t>
+          <t>__EMOJI__</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -1645,7 +1645,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>E711</t>
+          <t>E713</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Refs='__CTRL__'</t>
+          <t>Refs='   '</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>__CTRL__</t>
+          <t>   </t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1689,7 +1689,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>E712</t>
+          <t>E714</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1699,14 +1699,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Refs='__EMOJI__'</t>
+          <t>AccountType=99</t>
         </is>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>7</v>
+        <v>99</v>
       </c>
       <c r="F29" t="n">
         <v>6</v>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>__EMOJI__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1733,7 +1733,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>E713</t>
+          <t>E715</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1743,14 +1743,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Refs='   '</t>
+          <t>AccountType=-1</t>
         </is>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>7</v>
+        <v>-1</v>
       </c>
       <c r="F30" t="n">
         <v>6</v>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>   </t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -1777,7 +1777,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>E714</t>
+          <t>E716</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1787,14 +1787,16 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AccountType=99</t>
+          <t>AccountType='abc'</t>
         </is>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="E31" t="n">
-        <v>99</v>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
       </c>
       <c r="F31" t="n">
         <v>6</v>
@@ -1821,7 +1823,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>E715</t>
+          <t>E717</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1831,14 +1833,16 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AccountType=-1</t>
+          <t>AccountType='__MAXINT__'</t>
         </is>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="E32" t="n">
-        <v>-1</v>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>__MAXINT__</t>
+        </is>
       </c>
       <c r="F32" t="n">
         <v>6</v>
@@ -1865,7 +1869,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>E716</t>
+          <t>E718</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1875,7 +1879,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AccountType='abc'</t>
+          <t>AccountType='__HUGE__'</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1883,7 +1887,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>abc</t>
+          <t>__HUGE__</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -1911,7 +1915,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>E717</t>
+          <t>E719</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1921,19 +1925,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AccountType='__MAXINT__'</t>
+          <t>AccAtt=9</t>
         </is>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>__MAXINT__</t>
-        </is>
+      <c r="E34" t="n">
+        <v>7</v>
       </c>
       <c r="F34" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1957,7 +1959,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>E718</t>
+          <t>E720</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1967,19 +1969,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AccountType='__HUGE__'</t>
+          <t>AccAtt=-1</t>
         </is>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>__HUGE__</t>
-        </is>
+      <c r="E35" t="n">
+        <v>7</v>
       </c>
       <c r="F35" t="n">
-        <v>6</v>
+        <v>-1</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2003,7 +2003,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>E719</t>
+          <t>E721</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AccAtt=9</t>
+          <t>AccAtt='abc'</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2022,8 +2022,10 @@
       <c r="E36" t="n">
         <v>7</v>
       </c>
-      <c r="F36" t="n">
-        <v>9</v>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2047,7 +2049,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>E720</t>
+          <t>E722</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2057,7 +2059,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AccAtt=-1</t>
+          <t>FAccount=''</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2067,13 +2069,9 @@
         <v>7</v>
       </c>
       <c r="F37" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>010100011300</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
         <v>1</v>
       </c>
@@ -2091,7 +2089,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>E721</t>
+          <t>E723</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2101,7 +2099,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AccAtt='abc'</t>
+          <t>FAccount='__LONG__'</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2110,14 +2108,12 @@
       <c r="E38" t="n">
         <v>7</v>
       </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>abc</t>
-        </is>
+      <c r="F38" t="n">
+        <v>6</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>010100011300</t>
+          <t>__LONG__</t>
         </is>
       </c>
       <c r="H38" t="n">
@@ -2137,7 +2133,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>E722</t>
+          <t>E724</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2147,7 +2143,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>FAccount=''</t>
+          <t>FAccount='__CTRL__'</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2159,7 +2155,11 @@
       <c r="F39" t="n">
         <v>6</v>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>__CTRL__</t>
+        </is>
+      </c>
       <c r="H39" t="n">
         <v>1</v>
       </c>
@@ -2177,7 +2177,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>E723</t>
+          <t>E725</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>FAccount='__LONG__'</t>
+          <t>FAccount='__SQL__'</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>__LONG__</t>
+          <t>__SQL__</t>
         </is>
       </c>
       <c r="H40" t="n">
@@ -2221,17 +2221,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>E724</t>
+          <t>D900</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>destroy</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>FAccount='__CTRL__'</t>
+          <t>Refs='__LONG__'</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>__CTRL__</t>
+          <t>010100011300</t>
         </is>
       </c>
       <c r="H41" t="n">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__LONG__</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -2265,17 +2265,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>E725</t>
+          <t>D901</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>destroy</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>FAccount='__SQL__'</t>
+          <t>Refs='__REFS_MANY__'</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2289,7 +2289,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>__SQL__</t>
+          <t>010100011300</t>
         </is>
       </c>
       <c r="H42" t="n">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__REFS_MANY__</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -2309,7 +2309,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>D900</t>
+          <t>D902</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2319,7 +2319,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Refs='__LONG__'</t>
+          <t>Refs='__REFS_DUP__'</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>__LONG__</t>
+          <t>__REFS_DUP__</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2353,7 +2353,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>D901</t>
+          <t>D903</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Refs='__REFS_MANY__'</t>
+          <t>Refs='__REFS_SPACE__'</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>__REFS_MANY__</t>
+          <t>__REFS_SPACE__</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2397,7 +2397,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>D902</t>
+          <t>D904</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2407,7 +2407,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Refs='__REFS_DUP__'</t>
+          <t>Refs='__REFS_SQL__'</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>__REFS_DUP__</t>
+          <t>__REFS_SQL__</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2441,7 +2441,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>D903</t>
+          <t>D905</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Refs='__REFS_SPACE__'</t>
+          <t>Refs='__REFS_EMOJI__'</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>__REFS_SPACE__</t>
+          <t>__REFS_EMOJI__</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -2485,7 +2485,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>D904</t>
+          <t>D906</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Refs='__REFS_SQL__'</t>
+          <t>Refs='__CTRL__'</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>__REFS_SQL__</t>
+          <t>__CTRL__</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -2529,7 +2529,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>D905</t>
+          <t>D907</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Refs='__REFS_EMOJI__'</t>
+          <t>Refs='__SQL__'</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>__REFS_EMOJI__</t>
+          <t>__SQL__</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2573,7 +2573,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>D906</t>
+          <t>D908</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Refs='__CTRL__'</t>
+          <t>Refs='__EMOJI2__'</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>__CTRL__</t>
+          <t>__EMOJI2__</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -2617,7 +2617,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>D907</t>
+          <t>D909</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Refs='__SQL__'</t>
+          <t>Mode='__HUGE__'</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2644,12 +2644,14 @@
           <t>010100011300</t>
         </is>
       </c>
-      <c r="H50" t="n">
-        <v>1</v>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>__HUGE__</t>
+        </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>__SQL__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2661,7 +2663,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>D908</t>
+          <t>D910</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2671,7 +2673,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Refs='__EMOJI2__'</t>
+          <t>Mode='__SCI__'</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2688,12 +2690,14 @@
           <t>010100011300</t>
         </is>
       </c>
-      <c r="H51" t="n">
-        <v>1</v>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>__SCI__</t>
+        </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>__EMOJI2__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -2705,7 +2709,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>D909</t>
+          <t>D911</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2715,7 +2719,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Mode='__HUGE__'</t>
+          <t>Mode='__FLOATINF__'</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -2734,7 +2738,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>__HUGE__</t>
+          <t>__FLOATINF__</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -2751,7 +2755,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>D910</t>
+          <t>D912</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2761,7 +2765,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Mode='__SCI__'</t>
+          <t>Mode='__FLOATNAN__'</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2780,7 +2784,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>__SCI__</t>
+          <t>__FLOATNAN__</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -2797,7 +2801,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>D911</t>
+          <t>D913</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2807,7 +2811,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Mode='__FLOATINF__'</t>
+          <t>Mode='__NEG__'</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -2826,7 +2830,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>__FLOATINF__</t>
+          <t>__NEG__</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -2843,7 +2847,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>D912</t>
+          <t>D914</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2853,7 +2857,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Mode='__FLOATNAN__'</t>
+          <t>FAccount='__LONG10__'</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -2867,13 +2871,11 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>010100011300</t>
-        </is>
-      </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>__FLOATNAN__</t>
-        </is>
+          <t>__LONG10__</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>1</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -2889,7 +2891,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>D913</t>
+          <t>D915</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2899,7 +2901,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Mode='__NEG__'</t>
+          <t>FAccount='__LONG100__'</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -2913,13 +2915,11 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>010100011300</t>
-        </is>
-      </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>__NEG__</t>
-        </is>
+          <t>__LONG100__</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>1</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
@@ -2935,7 +2935,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>D914</t>
+          <t>D916</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>FAccount='__LONG10__'</t>
+          <t>FAccount='__CTRL__'</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>__LONG10__</t>
+          <t>__CTRL__</t>
         </is>
       </c>
       <c r="H57" t="n">
@@ -2979,7 +2979,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>D915</t>
+          <t>D917</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>FAccount='__LONG100__'</t>
+          <t>FAccount='__NULLBYTE__'</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -3003,7 +3003,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>__LONG100__</t>
+          <t>__NULLBYTE__</t>
         </is>
       </c>
       <c r="H58" t="n">
@@ -3023,7 +3023,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>D916</t>
+          <t>D918</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3033,7 +3033,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>FAccount='__CTRL__'</t>
+          <t>FAccount='__SQL__'</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>__CTRL__</t>
+          <t>__SQL__</t>
         </is>
       </c>
       <c r="H59" t="n">
@@ -3067,7 +3067,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>D917</t>
+          <t>D919</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3077,7 +3077,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>FAccount='__NULLBYTE__'</t>
+          <t>FAccount='__XSS__'</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>__NULLBYTE__</t>
+          <t>__XSS__</t>
         </is>
       </c>
       <c r="H60" t="n">
@@ -3111,7 +3111,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>D918</t>
+          <t>D920</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>FAccount='__SQL__'</t>
+          <t>FAccount='__EMOJI2__'</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>__SQL__</t>
+          <t>__EMOJI2__</t>
         </is>
       </c>
       <c r="H61" t="n">
@@ -3155,7 +3155,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>D919</t>
+          <t>D921</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>FAccount='__XSS__'</t>
+          <t>FAccount='__JSON__'</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>__XSS__</t>
+          <t>__JSON__</t>
         </is>
       </c>
       <c r="H62" t="n">
@@ -3199,7 +3199,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>D920</t>
+          <t>D922</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3209,21 +3209,23 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>FAccount='__EMOJI2__'</t>
+          <t>AccountType='__HUGE__'</t>
         </is>
       </c>
       <c r="D63" t="n">
         <v>0</v>
       </c>
-      <c r="E63" t="n">
-        <v>7</v>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>__HUGE__</t>
+        </is>
       </c>
       <c r="F63" t="n">
         <v>6</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>__EMOJI2__</t>
+          <t>010100011300</t>
         </is>
       </c>
       <c r="H63" t="n">
@@ -3243,7 +3245,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>D921</t>
+          <t>D923</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3253,21 +3255,23 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>FAccount='__JSON__'</t>
+          <t>AccountType='__SCI__'</t>
         </is>
       </c>
       <c r="D64" t="n">
         <v>0</v>
       </c>
-      <c r="E64" t="n">
-        <v>7</v>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>__SCI__</t>
+        </is>
       </c>
       <c r="F64" t="n">
         <v>6</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>__JSON__</t>
+          <t>010100011300</t>
         </is>
       </c>
       <c r="H64" t="n">
@@ -3287,7 +3291,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>D922</t>
+          <t>D300</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3297,16 +3301,16 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>AccountType='__HUGE__'</t>
-        </is>
-      </c>
-      <c r="D65" t="n">
-        <v>0</v>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>__HUGE__</t>
-        </is>
+          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>7</v>
       </c>
       <c r="F65" t="n">
         <v>6</v>
@@ -3321,7 +3325,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__LONG__</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3333,7 +3337,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>D923</t>
+          <t>D301</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3343,16 +3347,16 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>AccountType='__SCI__'</t>
-        </is>
-      </c>
-      <c r="D66" t="n">
-        <v>0</v>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>__SCI__</t>
-        </is>
+          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>7</v>
       </c>
       <c r="F66" t="n">
         <v>6</v>
@@ -3367,7 +3371,7 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__REFS_MANY__</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3379,7 +3383,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>D300</t>
+          <t>D302</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3389,7 +3393,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
+          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3413,7 +3417,7 @@
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>__LONG__</t>
+          <t>__SQL__</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
@@ -3425,7 +3429,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>D301</t>
+          <t>D303</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3435,7 +3439,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
+          <t>destroy 账号010100011300 注入Mode=99</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3455,11 +3459,11 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>__REFS_MANY__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
@@ -3471,7 +3475,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>D302</t>
+          <t>D304</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3481,7 +3485,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
+          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3497,7 +3501,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>010100011300</t>
+          <t>__CTRL__</t>
         </is>
       </c>
       <c r="H69" t="n">
@@ -3505,7 +3509,7 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>__SQL__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
@@ -3517,7 +3521,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>D303</t>
+          <t>D305</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3527,7 +3531,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Mode=99</t>
+          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3535,8 +3539,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E70" t="n">
-        <v>7</v>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>__HUGE__</t>
+        </is>
       </c>
       <c r="F70" t="n">
         <v>6</v>
@@ -3547,7 +3553,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
@@ -3563,7 +3569,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>D304</t>
+          <t>D306</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3573,14 +3579,10 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
       <c r="E71" t="n">
         <v>7</v>
       </c>
@@ -3589,7 +3591,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>__CTRL__</t>
+          <t>010100011300</t>
         </is>
       </c>
       <c r="H71" t="n">
@@ -3597,7 +3599,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__LONG__</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -3609,7 +3611,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>D305</t>
+          <t>D307</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3619,18 +3621,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>__HUGE__</t>
-        </is>
+          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="n">
+        <v>7</v>
       </c>
       <c r="F72" t="n">
         <v>6</v>
@@ -3645,7 +3641,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__REFS_MANY__</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -3657,7 +3653,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>D306</t>
+          <t>D308</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3667,7 +3663,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
+          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -3687,7 +3683,7 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>__LONG__</t>
+          <t>__SQL__</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3699,7 +3695,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>D307</t>
+          <t>D309</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3709,7 +3705,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
+          <t>destroy 账号010100011300 注入Mode=99</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -3725,11 +3721,11 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>__REFS_MANY__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3741,7 +3737,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>D308</t>
+          <t>D310</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3751,7 +3747,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
+          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
@@ -3763,7 +3759,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>010100011300</t>
+          <t>__CTRL__</t>
         </is>
       </c>
       <c r="H75" t="n">
@@ -3771,7 +3767,7 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>__SQL__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3783,7 +3779,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>D309</t>
+          <t>D311</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3793,12 +3789,14 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Mode=99</t>
+          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
-      <c r="E76" t="n">
-        <v>7</v>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>__HUGE__</t>
+        </is>
       </c>
       <c r="F76" t="n">
         <v>6</v>
@@ -3809,7 +3807,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="I76" t="inlineStr">
         <is>
@@ -3825,7 +3823,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>D310</t>
+          <t>D312</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3835,10 +3833,14 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr"/>
+          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="E77" t="n">
         <v>7</v>
       </c>
@@ -3847,7 +3849,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>__CTRL__</t>
+          <t>010100011300</t>
         </is>
       </c>
       <c r="H77" t="n">
@@ -3855,7 +3857,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__LONG__</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -3867,7 +3869,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>D311</t>
+          <t>D313</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3877,14 +3879,16 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>__HUGE__</t>
-        </is>
+          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>7</v>
       </c>
       <c r="F78" t="n">
         <v>6</v>
@@ -3899,7 +3903,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__REFS_MANY__</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -3911,7 +3915,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>D312</t>
+          <t>D314</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3921,7 +3925,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
+          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3945,7 +3949,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>__LONG__</t>
+          <t>__SQL__</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -3957,7 +3961,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>D313</t>
+          <t>D315</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3967,7 +3971,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
+          <t>destroy 账号010100011300 注入Mode=99</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3987,11 +3991,11 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>__REFS_MANY__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -4003,7 +4007,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>D314</t>
+          <t>D316</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4013,7 +4017,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
+          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4029,7 +4033,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>010100011300</t>
+          <t>__CTRL__</t>
         </is>
       </c>
       <c r="H81" t="n">
@@ -4037,7 +4041,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>__SQL__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -4049,7 +4053,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>D315</t>
+          <t>D317</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4059,7 +4063,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Mode=99</t>
+          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4067,8 +4071,10 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E82" t="n">
-        <v>7</v>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>__HUGE__</t>
+        </is>
       </c>
       <c r="F82" t="n">
         <v>6</v>
@@ -4079,7 +4085,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="I82" t="inlineStr">
         <is>
@@ -4095,7 +4101,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>D316</t>
+          <t>D318</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4105,23 +4111,23 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
+          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E83" t="n">
         <v>7</v>
       </c>
       <c r="F83" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>__CTRL__</t>
+          <t>010100011300</t>
         </is>
       </c>
       <c r="H83" t="n">
@@ -4129,7 +4135,7 @@
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__LONG__</t>
         </is>
       </c>
       <c r="J83" t="inlineStr">
@@ -4141,7 +4147,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>D317</t>
+          <t>D319</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4151,21 +4157,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
+          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>__HUGE__</t>
-        </is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>7</v>
       </c>
       <c r="F84" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -4177,7 +4181,7 @@
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__REFS_MANY__</t>
         </is>
       </c>
       <c r="J84" t="inlineStr">
@@ -4189,7 +4193,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>D318</t>
+          <t>D320</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4199,7 +4203,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
+          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4223,7 +4227,7 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>__LONG__</t>
+          <t>__SQL__</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -4235,7 +4239,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>D319</t>
+          <t>D321</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4245,7 +4249,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
+          <t>destroy 账号010100011300 注入Mode=99</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4265,11 +4269,11 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>__REFS_MANY__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -4281,7 +4285,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>D320</t>
+          <t>D322</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4291,7 +4295,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
+          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4307,7 +4311,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>010100011300</t>
+          <t>__CTRL__</t>
         </is>
       </c>
       <c r="H87" t="n">
@@ -4315,7 +4319,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>__SQL__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -4327,7 +4331,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>D321</t>
+          <t>D323</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4337,7 +4341,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Mode=99</t>
+          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4345,8 +4349,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E88" t="n">
-        <v>7</v>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>__HUGE__</t>
+        </is>
       </c>
       <c r="F88" t="n">
         <v>0</v>
@@ -4357,7 +4363,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
@@ -4373,7 +4379,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>D322</t>
+          <t>D324</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4383,7 +4389,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
+          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4392,14 +4398,14 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="F89" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>__CTRL__</t>
+          <t>010100011300</t>
         </is>
       </c>
       <c r="H89" t="n">
@@ -4407,7 +4413,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__LONG__</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -4419,7 +4425,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>D323</t>
+          <t>D325</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4429,7 +4435,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
+          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4437,13 +4443,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>__HUGE__</t>
-        </is>
+      <c r="E90" t="n">
+        <v>1</v>
       </c>
       <c r="F90" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -4455,7 +4459,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__REFS_MANY__</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -4467,7 +4471,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>D324</t>
+          <t>D326</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4477,7 +4481,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
+          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4501,7 +4505,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>__LONG__</t>
+          <t>__SQL__</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -4513,7 +4517,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>D325</t>
+          <t>D327</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4523,7 +4527,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
+          <t>destroy 账号010100011300 注入Mode=99</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -4543,11 +4547,11 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>__REFS_MANY__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -4559,7 +4563,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>D326</t>
+          <t>D328</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4569,7 +4573,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
+          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -4585,7 +4589,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>010100011300</t>
+          <t>__CTRL__</t>
         </is>
       </c>
       <c r="H93" t="n">
@@ -4593,7 +4597,7 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>__SQL__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -4605,7 +4609,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>D327</t>
+          <t>D329</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4615,7 +4619,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Mode=99</t>
+          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -4623,8 +4627,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E94" t="n">
-        <v>1</v>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>__HUGE__</t>
+        </is>
       </c>
       <c r="F94" t="n">
         <v>6</v>
@@ -4635,7 +4641,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="I94" t="inlineStr">
         <is>
@@ -4651,7 +4657,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>D328</t>
+          <t>D330</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4661,7 +4667,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
+          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -4673,11 +4679,11 @@
         <v>1</v>
       </c>
       <c r="F95" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>__CTRL__</t>
+          <t>010100011300</t>
         </is>
       </c>
       <c r="H95" t="n">
@@ -4685,7 +4691,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__LONG__</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -4697,7 +4703,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>D329</t>
+          <t>D331</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4707,7 +4713,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
+          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -4715,13 +4721,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>__HUGE__</t>
-        </is>
+      <c r="E96" t="n">
+        <v>1</v>
       </c>
       <c r="F96" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -4733,7 +4737,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__REFS_MANY__</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -4745,7 +4749,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>D330</t>
+          <t>D332</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4755,7 +4759,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__LONG__</t>
+          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -4779,7 +4783,7 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>__LONG__</t>
+          <t>__SQL__</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
@@ -4791,7 +4795,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>D331</t>
+          <t>D333</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4801,7 +4805,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__REFS_MANY__</t>
+          <t>destroy 账号010100011300 注入Mode=99</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -4821,11 +4825,11 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>__REFS_MANY__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
@@ -4837,7 +4841,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>D332</t>
+          <t>D334</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4847,7 +4851,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Refs=__SQL__</t>
+          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -4863,7 +4867,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>010100011300</t>
+          <t>__CTRL__</t>
         </is>
       </c>
       <c r="H99" t="n">
@@ -4871,7 +4875,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>__SQL__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -4883,7 +4887,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>D333</t>
+          <t>D335</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4893,7 +4897,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入Mode=99</t>
+          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -4901,8 +4905,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E100" t="n">
-        <v>1</v>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>__HUGE__</t>
+        </is>
       </c>
       <c r="F100" t="n">
         <v>0</v>
@@ -4913,7 +4919,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="I100" t="inlineStr">
         <is>
@@ -4929,7 +4935,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>D334</t>
+          <t>D336</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4939,7 +4945,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入FAccount=__CTRL__</t>
+          <t>destroy 账号 010100011300 注入Refs=__LONG__</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -4948,14 +4954,14 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F101" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>__CTRL__</t>
+          <t xml:space="preserve"> 010100011300</t>
         </is>
       </c>
       <c r="H101" t="n">
@@ -4963,7 +4969,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__LONG__</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -4975,7 +4981,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>D335</t>
+          <t>D337</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -4985,7 +4991,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>destroy 账号010100011300 注入AccountType=__HUGE__</t>
+          <t>destroy 账号 010100011300 注入Refs=__REFS_MANY__</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -4993,17 +4999,15 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>__HUGE__</t>
-        </is>
+      <c r="E102" t="n">
+        <v>7</v>
       </c>
       <c r="F102" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>010100011300</t>
+          <t xml:space="preserve"> 010100011300</t>
         </is>
       </c>
       <c r="H102" t="n">
@@ -5011,7 +5015,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>__REF1__</t>
+          <t>__REFS_MANY__</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -5023,7 +5027,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>D336</t>
+          <t>D338</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -5033,7 +5037,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>destroy 账号 010100011300 注入Refs=__LONG__</t>
+          <t>destroy 账号 010100011300 注入Refs=__SQL__</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5057,7 +5061,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>__LONG__</t>
+          <t>__SQL__</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -5069,7 +5073,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>D337</t>
+          <t>D339</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -5079,7 +5083,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>destroy 账号 010100011300 注入Refs=__REFS_MANY__</t>
+          <t>destroy 账号 010100011300 注入Mode=99</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5099,11 +5103,11 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>1</v>
+        <v>99</v>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>__REFS_MANY__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -5115,7 +5119,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>D338</t>
+          <t>D340</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -5125,7 +5129,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>destroy 账号 010100011300 注入Refs=__SQL__</t>
+          <t>destroy 账号 010100011300 注入FAccount=__CTRL__</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -5141,7 +5145,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 010100011300</t>
+          <t>__CTRL__</t>
         </is>
       </c>
       <c r="H105" t="n">
@@ -5149,7 +5153,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>__SQL__</t>
+          <t>__REF1__</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -5161,7 +5165,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>D339</t>
+          <t>D341</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5171,7 +5175,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>destroy 账号 010100011300 注入Mode=99</t>
+          <t>destroy 账号 010100011300 注入AccountType=__HUGE__</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -5179,8 +5183,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E106" t="n">
-        <v>7</v>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>__HUGE__</t>
+        </is>
       </c>
       <c r="F106" t="n">
         <v>6</v>
@@ -5191,7 +5197,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>99</v>
+        <v>1</v>
       </c>
       <c r="I106" t="inlineStr">
         <is>
@@ -5199,100 +5205,6 @@
         </is>
       </c>
       <c r="J106" t="inlineStr">
-        <is>
-          <t>主用例：模板行，字段值勿改</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>D340</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>destroy</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>destroy 账号 010100011300 注入FAccount=__CTRL__</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E107" t="n">
-        <v>7</v>
-      </c>
-      <c r="F107" t="n">
-        <v>6</v>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>__CTRL__</t>
-        </is>
-      </c>
-      <c r="H107" t="n">
-        <v>1</v>
-      </c>
-      <c r="I107" t="inlineStr">
-        <is>
-          <t>__REF1__</t>
-        </is>
-      </c>
-      <c r="J107" t="inlineStr">
-        <is>
-          <t>主用例：模板行，字段值勿改</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>D341</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>destroy</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>destroy 账号 010100011300 注入AccountType=__HUGE__</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>__HUGE__</t>
-        </is>
-      </c>
-      <c r="F108" t="n">
-        <v>6</v>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> 010100011300</t>
-        </is>
-      </c>
-      <c r="H108" t="n">
-        <v>1</v>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>__REF1__</t>
-        </is>
-      </c>
-      <c r="J108" t="inlineStr">
         <is>
           <t>主用例：模板行，字段值勿改</t>
         </is>

</xml_diff>